<commit_message>
Save library recording Session 12/10/2026, 8:22:44 am - 057e5aa5-fcd1-4642-8673-a96b499e0887 - 2026-10-11T21:29:12.536002Z
</commit_message>
<xml_diff>
--- a/library/projects/a8107955-5370-4125-bfc0-813060e10786/recordings/057e5aa5-fcd1-4642-8673-a96b499e0887/resources/azure-devops.xlsx
+++ b/library/projects/a8107955-5370-4125-bfc0-813060e10786/recordings/057e5aa5-fcd1-4642-8673-a96b499e0887/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,560 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://login.microsoftonline.com/74512bd2-de5d-4870-83ee-50eebf992b45/oauth2/authorize?client_id=00000015-0000-0000-c000-000000000000&amp;response_type=code%20id_token&amp;scope=openid%20profile&amp;state=OpenIdConnect.AuthenticationProperties%3DAQAAANCMnd8BFdERjHoAwE_Cl-sBAAAACtQKQ4Qtkk-zuqZ4Dv9DWwAAAAACAAAAAAAQZgAAAAEAACAAAABEo21UoRzOikQ6xy530x73fjrP-WtdCbgSlunJT97c7AAAAAAOgAAAAAIAACAAAADmlVDv7fikZaQiNtHT6i9sTdOJANjIyh6XAnFYHpks8HAAAABXoU-nCmD9r92iij_RP0sQuG_W1gOnFDRk2EvbDZIXkCtXKzivKvpR_bhFkwPFBkJ…</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://login.microsoftonline.com/74512bd2-de5d-4870-83ee-50eebf992b45/oauth2/authorize?client_id=00000015-0000-0000-c000-000000000000&amp;response_type=code%20id_token&amp;scope=openid%20profile&amp;state=OpenIdConnect.AuthenticationProperties%3DAQAAANCMnd8BFdERjHoAwE_Cl-sBAAAACtQKQ4Qtkk-zuqZ4Dv9DWwAAAAACAAAAAAAQZgAAAAEAACAAAABEo21UoRzOikQ6xy530x73fjrP-WtdCbgSlunJT97c7AAAAAAOgAAAAAIAACAAAADmlVDv7fikZaQiNtHT6i9sTdOJANjIyh6XAnFYHpks8HAAAABXoU-nCmD9r92iij_RP0sQuG_W1gOnFDRk2EvbDZIXkCtXKzivKvpR_bhFkwPFBkJ1AefGcXV6xvOv02aefo3D7Jwrn0yFr4HFpo0UAW3B7G61B9m0HQQUn3oUDrKg4FrJ-bfDhrfDyYpZ_zE0FrG_QAAAAG8Zm6PvsF4hf9MAyIt-6Oocn6jtYSXwa-UJt5htKyJRRMjroahaYYyxdw3iVIEtqc7hEjc-UioY6qH3IpeL1U0%26RedirectTo%3Dhttps%253A%252F%252Fharrisfarm-uat.sandbox.operations.dynamics.com%252F&amp;response_mode=form_post&amp;nonce=639273506181049180.M2IzM2QwOTEtMzJhZi00NWU3LTg0ZjEtOWE0ODk5NjJhNDA0NjBjZTk0YzEtOTRjZC00ZTc3LTk0ZWYtMWZhN2NkNDlhZjhm&amp;redirect_uri=https%3A%2F%2Fgw.au-il102.gateway.prod.island.powerapps.com%2Freplyurl%2Fv1&amp;max_age=86400&amp;x-client-SKU=ID_NET472&amp;x-client-ver=8.3.0.0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click Enter your email, phone, or Skype.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "#i0116", "x": 362, "y": 249, "text": "Enter your email, phone, or Skype.", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Type: {{D365_Login_ID}}</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{{D365_Login_ID}}</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "#i0116"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Press Tab</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Click Next</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"primary": "#idSIButton9", "x": 647, "y": 380, "text": "Next", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>step-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Click Enter the password for ratta@harrisfarm.com.au</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"primary": "#i0118", "x": 360, "y": 299, "text": "Enter the password for ratta@harrisfarm.com.au", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>step-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Type: {{D365_login_Pass}}</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{{D365_login_Pass}}</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"primary": "#i0118"}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>step-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Press Tab</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tab</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>step-008.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Click Sign in</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"primary": "#idSIButton9", "x": 640, "y": 433, "text": "Sign in", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>step-009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Click ratta@harrisfarm.com.au
+Let's keep your account secure
+We'll help you set up ano</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"primary": "#lightbox", "x": 640, "y": 433, "text": "ratta@harrisfarm.com.au\nLet's keep your account secure\nWe'll help you set up ano", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>step-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Click Not now</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"primary": "#skipMfaRegistrationLink", "x": 358, "y": 362, "text": "Not now", "tag": "a"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>step-011.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Click Yes</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"primary": "#idSIButton9", "x": 622, "y": 434, "text": "Yes", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>step-012.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Click Order</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"primary": "#GridHeader_Num_3_0_header &gt; div:nth-of-type(1)", "x": 444, "y": 413, "text": "Order", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>step-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Click Sort largest to smallest</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"primary": "#__Descending_GridHeader_Num_label", "x": 465, "y": 224, "text": "Sort largest to smallest", "tag": "span"}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>step-014.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Click Order</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"primary": "#GridHeader_Num_3_0_header &gt; div:nth-of-type(1)", "x": 441, "y": 412, "text": "Order", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>step-015.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Click Filter field: Order, operator: is equal to</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{"primary": "#__FilterField_GridHeader_Num_Num_Input_0_0_input", "x": 447, "y": 332, "text": "Filter field: Order, operator: is equal to", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>step-016.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Type: 91020262</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>91020262</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{"primary": "#__FilterField_GridHeader_Num_Num_Input_0_0_input"}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>step-017.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Click Apply</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{"primary": "#__GridHeader_Num_ApplyFilters_label", "x": 434, "y": 370, "text": "Apply", "tag": "span"}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>step-018.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Session 12/10/2026, 8:22:44 am</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Click 91020262</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{"primary": "#GridHeader_Num_3_0_0_input", "x": 442, "y": 448, "text": "91020262", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>step-019.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>